<commit_message>
adding PDF for coloc mini-plot panel for fig. 7
</commit_message>
<xml_diff>
--- a/processed-data/eQTL/coloc/coloc_results.xlsx
+++ b/processed-data/eQTL/coloc/coloc_results.xlsx
@@ -50,10 +50,10 @@
     <t xml:space="preserve">risk_SNP_GWAS</t>
   </si>
   <si>
-    <t xml:space="preserve">SCZD_DGE_layer_adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCZD_DGE_layer_adjusted_p05</t>
+    <t xml:space="preserve">SCZD_DEG_layer_adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCZD_DEG_layer_adjusted_p05</t>
   </si>
   <si>
     <t xml:space="preserve">eQTL_independent</t>

</xml_diff>